<commit_message>
Changes & new Required files Added
</commit_message>
<xml_diff>
--- a/backend/students.xlsx
+++ b/backend/students.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,7 +461,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>supriyam.2410@gmail.com</t>
+          <t>supriya.2410@gmail.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -503,12 +503,76 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>9999999999</t>
+          <t>9988908765</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>rajesh@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sangli</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4829292929</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Barkha</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>barkha@gmail.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>7890234487</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Female</t>
         </is>
       </c>
     </row>

</xml_diff>